<commit_message>
zippped, doc bugs fixed
</commit_message>
<xml_diff>
--- a/sample_apps/dst_stn_ja/dst_knowledge_ja.xlsx
+++ b/sample_apps/dst_stn_ja/dst_knowledge_ja.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nakano\system\dialbb\dialbb-next\sample_apps\dst_stn_ja\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86709119-3ECA-43C5-B8C0-1ACE2C1CE480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA23D51E-77AF-496E-BF99-A031E9DDC325}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28605" yWindow="-195" windowWidth="29190" windowHeight="15870" activeTab="1" xr2:uid="{C3566FB2-A815-41D8-9347-99D11DD601B4}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C3566FB2-A815-41D8-9347-99D11DD601B4}"/>
   </bookViews>
   <sheets>
     <sheet name="dialogues" sheetId="2" r:id="rId1"/>

</xml_diff>